<commit_message>
Invalidate dependents of moved manual spill caches
</commit_message>
<xml_diff>
--- a/tests/fixtures/manual_spill_cache/clear_child.xlsx
+++ b/tests/fixtures/manual_spill_cache/clear_child.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\pyOpenVBA\tests\fixtures\manual_spill_cache\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01FB3695-C801-4419-B0F4-0CFA6E1AEACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A28492B2-BD3E-496C-95AE-E5DAB334BFA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="7200" windowHeight="4545" xr2:uid="{14E9F74F-1BAC-41C2-83BA-62D91B513F2F}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="7200" windowHeight="4545" xr2:uid="{7863C38A-5E57-44AA-9F0A-CBAEC5AEEEB6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -504,7 +504,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F62B9E34-1B65-49C2-B7EF-CD36AAA3D3E3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F0EF13A-9625-4113-9C56-AF3453FA1650}">
   <dimension ref="B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -520,7 +520,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0A6FC05-3A7C-4D5D-970A-3353A4515D29}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8220D26-909A-478B-8633-0DB693D2DB71}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>